<commit_message>
Update extended test questions
</commit_message>
<xml_diff>
--- a/evaluation/test_questions_extended.xlsx
+++ b/evaluation/test_questions_extended.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/f1ad9b415b81f28d/Desktop/Master/WBH/3. Semester/Forschungsarbeit inkl. Fachseminar/text_to_sql_prototype/evaluation/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="31" documentId="11_AD4DB114E441178AC67DF40AF693DEDE693EDF18" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{0F6EF7E3-5774-4C0A-825F-192C1341B3A4}"/>
+  <xr:revisionPtr revIDLastSave="33" documentId="11_AD4DB114E441178AC67DF40AF693DEDE693EDF18" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{699DBD50-74C1-499E-9463-AA75F59E5EDE}"/>
   <bookViews>
-    <workbookView xWindow="1170" yWindow="1170" windowWidth="21600" windowHeight="11295" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-105" yWindow="0" windowWidth="14610" windowHeight="15585" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Tabelle1" sheetId="1" r:id="rId1"/>
@@ -45,15 +45,9 @@
     <t>L3</t>
   </si>
   <si>
-    <t>Which prioritized customer generated the highest net revenue from high-value products in completed Summer Sale orders?</t>
-  </si>
-  <si>
     <t>R3</t>
   </si>
   <si>
-    <t>Which VIP customer successfully purchased high-value products with a discount greater than 20%?</t>
-  </si>
-  <si>
     <t>How many completed Summer Sale orders were placed by customers from the Automation Segment?</t>
   </si>
   <si>
@@ -79,6 +73,12 @@
   </si>
   <si>
     <t>Q55</t>
+  </si>
+  <si>
+    <t>Which VIP customers ordered products with a discount greater than 20%?</t>
+  </si>
+  <si>
+    <t>Which customer from the Growth Market Segment generated the highest net revenue from completed Summer Sale orders?</t>
   </si>
 </sst>
 </file>
@@ -447,63 +447,63 @@
     </row>
     <row r="2" spans="1:4" ht="30" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="C2" s="3" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="D2" s="3" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
     </row>
     <row r="3" spans="1:4" ht="45" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="C3" s="3" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="D3" s="3" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
     </row>
-    <row r="4" spans="1:4" ht="45" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:4" ht="30" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>8</v>
+        <v>16</v>
       </c>
       <c r="C4" s="3" t="s">
         <v>5</v>
       </c>
       <c r="D4" s="3" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
     </row>
     <row r="5" spans="1:4" ht="60" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>6</v>
+        <v>17</v>
       </c>
       <c r="C5" s="3" t="s">
         <v>5</v>
       </c>
       <c r="D5" s="3" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
     </row>
     <row r="6" spans="1:4" ht="60" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="B6" s="2" t="s">
         <v>4</v>
@@ -512,7 +512,7 @@
         <v>5</v>
       </c>
       <c r="D6" s="3" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
     </row>
   </sheetData>

</xml_diff>